<commit_message>
fix: Define spec variables at top of scope to prevent ReferenceError and remove duplicates
</commit_message>
<xml_diff>
--- a/PU333_01_엔진_v11.0.xlsx
+++ b/PU333_01_엔진_v11.0.xlsx
@@ -4755,7 +4755,7 @@
       </c>
       <c r="B15" s="66" t="inlineStr">
         <is>
-          <t>성장판 프리패스상</t>
+          <t>【성장판 프리패스】 프로 지행상</t>
         </is>
       </c>
       <c r="C15" s="67" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="B16" s="66" t="inlineStr">
         <is>
-          <t>성장가능 가치주</t>
+          <t>【성장 우량주】 프레임 확장 유망주</t>
         </is>
       </c>
       <c r="C16" s="67" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B17" s="66" t="inlineStr">
         <is>
-          <t>불타오른 야생마</t>
+          <t>【과부하 야생마】 엔진 과열 패턴</t>
         </is>
       </c>
       <c r="C17" s="67" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="B18" s="66" t="inlineStr">
         <is>
-          <t>직진형 에너자이저</t>
+          <t>【직진형 에너자이저】 모범적 프레임</t>
         </is>
       </c>
       <c r="C18" s="67" t="inlineStr">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="B19" s="66" t="inlineStr">
         <is>
-          <t>성장계의 엄친아</t>
+          <t>【엄친아 성장 정석】 안정적 우량군</t>
         </is>
       </c>
       <c r="C19" s="67" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="B20" s="66" t="inlineStr">
         <is>
-          <t>이중생활 천재선수</t>
+          <t>【불꽃 소모 불나방】 야간 방전 패턴</t>
         </is>
       </c>
       <c r="C20" s="67" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="B21" s="66" t="inlineStr">
         <is>
-          <t>예민보스 모범생</t>
+          <t>【유리 위장 거인 유망주】 대사 단절형</t>
         </is>
       </c>
       <c r="C21" s="67" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="B22" s="66" t="inlineStr">
         <is>
-          <t>멘탈소심 거인</t>
+          <t>【쿠쿠다스 멘탈 거인】 불안정 성장군</t>
         </is>
       </c>
       <c r="C22" s="67" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="B23" s="66" t="inlineStr">
         <is>
-          <t>파업선언 장군님</t>
+          <t>【장군님의 파업 선언】 총체적 방해 패턴</t>
         </is>
       </c>
       <c r="C23" s="67" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="B24" s="66" t="inlineStr">
         <is>
-          <t>노력형 디젤엔진</t>
+          <t>【노력형 디젤 엔진】 후천적 강자</t>
         </is>
       </c>
       <c r="C24" s="67" t="inlineStr">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B25" s="66" t="inlineStr">
         <is>
-          <t>뷔페 환영 보일러</t>
+          <t>【뷔페 환영 보일러】 영양 폭발형</t>
         </is>
       </c>
       <c r="C25" s="67" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B26" s="66" t="inlineStr">
         <is>
-          <t>폭풍흡수 먹방러</t>
+          <t>【폭풍 흡수 야식 요정】 비만 위험군</t>
         </is>
       </c>
       <c r="C26" s="67" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="B27" s="66" t="inlineStr">
         <is>
-          <t>바른생활 부반장</t>
+          <t>【바른 생활 캡틴】 규율형 표준군</t>
         </is>
       </c>
       <c r="C27" s="67" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>이세계의 무게중심</t>
+          <t>【평화주의 프로평범러】 일반 아동 표준</t>
         </is>
       </c>
       <c r="C28" s="67" t="inlineStr">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="B29" s="66" t="inlineStr">
         <is>
-          <t>여유만만 도련님</t>
+          <t>【침대 일체형 늘보】 활동 결핍형</t>
         </is>
       </c>
       <c r="C29" s="67" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B30" s="66" t="inlineStr">
         <is>
-          <t>안절부절 바른생활</t>
+          <t>【속 타는 바른 생활이】 소심한 모범생</t>
         </is>
       </c>
       <c r="C30" s="67" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="B31" s="66" t="inlineStr">
         <is>
-          <t>내일향한 숨고르기</t>
+          <t>【훈련 과다 슬럼프 정체기】 선수 다수 분포</t>
         </is>
       </c>
       <c r="C31" s="67" t="inlineStr">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="B32" s="66" t="inlineStr">
         <is>
-          <t>비상임박 유망주</t>
+          <t>【잔소리 유발 유망주】 악순환 정체군</t>
         </is>
       </c>
       <c r="C32" s="67" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="B33" s="66" t="inlineStr">
         <is>
-          <t>대기만성 반전매력</t>
+          <t>【대기만성 반전 유망주】 스펀지 도토리</t>
         </is>
       </c>
       <c r="C33" s="67" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="B34" s="66" t="inlineStr">
         <is>
-          <t>알짜배기 깡다구</t>
+          <t>【알짜배기 도토리】 추격형 소형마</t>
         </is>
       </c>
       <c r="C34" s="67" t="inlineStr">
@@ -5295,7 +5295,7 @@
       </c>
       <c r="B35" s="66" t="inlineStr">
         <is>
-          <t>엔진빵빵 클래식카</t>
+          <t>【엔진만 좋은 클래식카】 자원 낭비형</t>
         </is>
       </c>
       <c r="C35" s="67" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="B36" s="66" t="inlineStr">
         <is>
-          <t>의지만렙 작은거인</t>
+          <t>【의지 만렙 스몰 자이언트】 신체 하드캐리</t>
         </is>
       </c>
       <c r="C36" s="67" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="B37" s="66" t="inlineStr">
         <is>
-          <t>작은고추 매운맛</t>
+          <t>【작지만 매운 청양고추】 이번 민우 선수</t>
         </is>
       </c>
       <c r="C37" s="67" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B38" s="66" t="inlineStr">
         <is>
-          <t>출동준비 비행기</t>
+          <t>【성장 정지 비행기】 난기류 위험군</t>
         </is>
       </c>
       <c r="C38" s="67" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="B39" s="66" t="inlineStr">
         <is>
-          <t>상큼발랄 팅커벨</t>
+          <t>【정신 승리 요정】 눈물겨운 모범생</t>
         </is>
       </c>
       <c r="C39" s="67" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B40" s="66" t="inlineStr">
         <is>
-          <t>우리동네 골목대장</t>
+          <t>【골골 골목대장】 면역 방전형</t>
         </is>
       </c>
       <c r="C40" s="67" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="B41" s="66" t="inlineStr">
         <is>
-          <t>무한성장 기대주</t>
+          <t>【귀하신 몸 집중 케어】 레드 라이트 위기</t>
         </is>
       </c>
       <c r="C41" s="67" t="inlineStr">

</xml_diff>